<commit_message>
readable headers and colour on the effect tab
</commit_message>
<xml_diff>
--- a/results/review/52_codes_review.xlsx
+++ b/results/review/52_codes_review.xlsx
@@ -3,23 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="the six that look wrong" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="by chapter" sheetId="3" state="visible" r:id="rId2"/>
-    <sheet name="the other 46" sheetId="5" state="visible" r:id="rId3"/>
-    <sheet name="accuracy effect" sheetId="6" state="visible" r:id="rId4"/>
+    <sheet name="by chapter" sheetId="3" state="visible" r:id="rId1"/>
+    <sheet name="the other 46" sheetId="5" state="visible" r:id="rId2"/>
+    <sheet name="accuracy effect" sheetId="8" state="visible" r:id="rId4"/>
+    <sheet name="the six that look wrong" sheetId="7" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'the other 46'!$A$1:$G$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'the other 46'!$A$1:$G$47</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="418">
   <si>
     <t>ICD-9-CM</t>
   </si>
@@ -1042,6 +1042,237 @@
   </si>
   <si>
     <t xml:space="preserve">SapBERT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICD-9-CM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICD-9-CM label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICD-9 chapter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proposed ICDA-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICDA-8 label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Justification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICDA-8 codes in that block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ClinicalBERT top cosine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank of proposed, ClinicalBERT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SapBERT top cosine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank of proposed, SapBERT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the co-occurrence data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">165</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malignant neoplasm of other and illdefined sites within the respiratory system and intrathoracic organs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 neoplasms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">163</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malignant neoplasm of other and unspecified respiratory organs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Its respiratory block stops at 163, other and unspecified respiratory organs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">160 malignant neoplasm of nose nasal cavities middle ear and accessory sinuses; 161 malignant neoplasm of larynx; 162 malignant neoplasm of trachea bronchus and lung; 163 malignant neoplasm of other and unspecified respiratory organs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">187 malignant neoplasm of other and unspecified male genital organs (0.965)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#4 of 858 (0.963)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">163 malignant neoplasm of other and unspecified respiratory organs (0.823)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1 of 858 (0.823)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">175</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malignant neoplasm of male breast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malignant neoplasm of breast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breast cancer is one code in ICDA-8, 174. Not split by sex.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">172 malignant melanoma of skin; 173 other malignant neoplasm of skin; 174 malignant neoplasm of breast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">174 malignant neoplasm of breast (0.988)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1 of 858 (0.988)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">174 malignant neoplasm of breast (0.774)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1 of 858 (0.774)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malignant neoplasm of uterus part unspecified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other malignant neoplasm of uterus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The uterus is split into 180 cervix, 181 chorionepithelioma and 182 other, so part unspecified goes to 182.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180 malignant neoplasm of cervix uteri; 181 chorionepithelioma; 182 other malignant neoplasm of uterus; 183 malignant neoplasm of ovary fallopian tube and broad ligament</t>
+  </si>
+  <si>
+    <t xml:space="preserve">149 malignant neoplasm of pharynx unspecified (0.985)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#39 of 858 (0.930)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">182 other malignant neoplasm of uterus (0.793)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1 of 858 (0.793)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">555</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regional enteritis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 digestive system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">563</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chronic enteritis and ulcerative colitis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional enteritis is a form of chronic enteritis, and 563 is the chronic one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">560 intestinal obstruction without mention of hernia; 561 gastroenteritis and colitis except ulcerative of noninfectious origin; 562 diverticula of intestine; 563 chronic enteritis and ulcerative colitis; 564 functional disorders of intestines; 565 anal fissure and fistula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">518 bronchiectasis (0.927)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#47 of 858 (0.910)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">563 chronic enteritis and ulcerative colitis (0.721)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1 of 858 (0.721)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other disorders of biliary tract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other diseases of gallbladder and biliary ducts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same number in both, and the same thing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574 cholelithiasis; 575 cholecystitis and cholangitis without mention of calculus; 576 other diseases of gallbladder and biliary ducts; 577 diseases of pancreas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">508 other diseases of upper respiratory tract (0.976)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#11 of 858 (0.951)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576 other diseases of gallbladder and biliary ducts (0.868)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1 of 858 (0.868)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">745</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bulbus cordis anomalies and anomalies of cardiac septal closure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 congenital anomalies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">746</t>
+  </si>
+  <si>
+    <t xml:space="preserve">congenital anomalies of heart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICD-9 745 is a heart defect and 746 is the only heart code in ICDA-8. ICDA-8 745 also exists but it is ear, face and neck, so the numbers do not line up between the two systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">743 other congenital anomalies of nervous system; 744 congenital anomalies of eye; 745 congenital anomalies of ear face and neck; 746 congenital anomalies of heart; 747 other congenital anomalies of circulatory system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">524 dentofacial anomalies including malocclusion (0.924)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#257 of 858 (0.867)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">745 congenital anomalies of ear face and neck (0.526)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#4 of 858 (0.509)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1 if the 52 are dropped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1 with the six fixes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1 change from including</t>
   </si>
 </sst>
 </file>
@@ -1069,7 +1300,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1084,6 +1315,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDF1E4"/>
       </patternFill>
     </fill>
   </fills>
@@ -1104,7 +1345,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1115,6 +1356,11 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1414,319 +1660,6 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="28.6640625" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="38.6640625" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="70.6640625" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="70.6640625" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="22.6640625" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="34.6640625" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="17.6640625" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="34.6640625" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="17.6640625" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="12.6640625" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="43.2" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" ht="43.2" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" ht="28.8" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" ht="43.2" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" ht="57.6" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" ht="28.8" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" ht="43.2" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
     <col min="1" max="1" width="42.6640625" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" hidden="0" customWidth="1"/>
@@ -1893,7 +1826,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -2995,508 +2928,847 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="34.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="28.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="38.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="70.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="70.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="34.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="17.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="34.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="17.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="12.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="14.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="8.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="30.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="14.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="14.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="14.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="15.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="13.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="17.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="15.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="13.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="13.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="10.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="9.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="8.71" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="10.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="16.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="15.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>334</v>
+      <c r="O1" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>0.999</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>331</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>244</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="5" t="n">
         <v>147</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="5" t="n">
         <v>87</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="5" t="n">
         <v>0.624</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="5" t="n">
         <v>0.737</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="5" t="n">
         <v>0.676</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="5" t="n">
         <v>0.51</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2" s="5" t="n">
         <v>0.702</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="5" t="n">
         <v>0.673</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2" s="5" t="n">
         <v>-0.026</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>0.999</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>331</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>167</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="5" t="n">
         <v>164</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="5" t="n">
         <v>0.663</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="5" t="n">
         <v>0.505</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="5" t="n">
         <v>0.573</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="5" t="n">
         <v>0.401</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3" s="5" t="n">
         <v>0.601</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="5" t="n">
         <v>0.57</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q3" s="5" t="n">
         <v>-0.028</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>0.999</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>331</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>227</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="5" t="n">
         <v>74</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="5" t="n">
         <v>104</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="5" t="n">
         <v>0.754</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="5" t="n">
         <v>0.686</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="5" t="n">
         <v>0.718</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="5" t="n">
         <v>0.56</v>
       </c>
-      <c r="O4" t="n">
+      <c r="O4" s="5" t="n">
         <v>0.718</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" s="5" t="n">
         <v>0.712</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="Q4" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.999</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>331</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>244</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="5" t="n">
         <v>149</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="5" t="n">
         <v>87</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="5" t="n">
         <v>0.621</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="5" t="n">
         <v>0.737</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="5" t="n">
         <v>0.674</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="5" t="n">
         <v>0.508</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="5" t="n">
         <v>0.671</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q5" s="5" t="n">
         <v>-0.026</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="6" t="n">
         <v>0.995</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="6" t="n">
         <v>269</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="6" t="n">
         <v>145</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="6" t="n">
         <v>0.65</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="6" t="n">
         <v>0.813</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="6" t="n">
         <v>0.722</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="6" t="n">
         <v>0.565</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="6" t="n">
         <v>0.765</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" s="6" t="n">
         <v>0.73</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6" s="6" t="n">
         <v>-0.043</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="6" t="n">
         <v>0.995</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="6" t="n">
         <v>246</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="6" t="n">
         <v>80</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="6" t="n">
         <v>0.755</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="6" t="n">
         <v>0.743</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="6" t="n">
         <v>0.749</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="6" t="n">
         <v>0.599</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O7" s="6" t="n">
         <v>0.8</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7" s="6" t="n">
         <v>0.757</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7" s="6" t="n">
         <v>-0.051</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="6" t="n">
         <v>0.995</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="6" t="n">
         <v>244</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="6" t="n">
         <v>73</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="6" t="n">
         <v>87</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="6" t="n">
         <v>0.77</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="6" t="n">
         <v>0.737</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="6" t="n">
         <v>0.753</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="6" t="n">
         <v>0.604</v>
       </c>
-      <c r="O8" t="n">
+      <c r="O8" s="6" t="n">
         <v>0.753</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P8" s="6" t="n">
         <v>0.746</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q8" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="6" t="n">
         <v>0.995</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="6" t="n">
         <v>331</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="6" t="n">
         <v>269</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="6" t="n">
         <v>145</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="6" t="n">
         <v>0.65</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="6" t="n">
         <v>0.813</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="6" t="n">
         <v>0.722</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="6" t="n">
         <v>0.565</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9" s="6" t="n">
         <v>0.765</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" s="6" t="n">
         <v>0.73</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q9" s="6" t="n">
         <v>-0.043</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="M2:M9">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="0.7"/>
+        <cfvo type="num" val="0.85"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K9">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="0.7"/>
+        <cfvo type="num" val="0.85"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L9">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="0.7"/>
+        <cfvo type="num" val="0.85"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N9">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="0.7"/>
+        <cfvo type="num" val="0.85"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>

</xml_diff>